<commit_message>
P5.15 Addendum 27: bring the author's corrected cost file onto this branch (SRP1_ESS.xlsx from 7ce1d1ab)
Author's decision (Addendum 27): data/SRP1/SharedESS/SRP1_ESS.xlsx at 7ce1d1ab ('Costs updated.',
2026-07-29, branch paper_revisions) is the corrected cost file. Brought onto this branch alone, by
path checkout from that commit, committed by name. Energy unit costs x1.25 relative to the file it
replaces; power costs, scenario weights and other sheets unchanged (Addendum 26 confirmations).
sha256 before 1458147446e9b70190465f42cef761af9cfd8b209e91035d858e2e63941d1414
sha256 after  e17bd5887e1d0738005ae17c3144593527081c9a0776e19cfaa50aafefe39cd6
It affects I(x) only; the oracle's Q(x) does not read it (Addendum 27), so evaluations already
committed stay valid.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/SRP1/SharedESS/SRP1_ESS.xlsx
+++ b/data/SRP1/SharedESS/SRP1_ESS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\Shared ESS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/micaelsimoes/PycharmProjects/shared-resources-planning/data/SRP1/SharedESS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80ED936D-F119-451E-A679-B6E072B7D176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C26F2DB-8A39-1E48-B60C-F64E7E7BA667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31920" yWindow="-11265" windowWidth="28800" windowHeight="15285" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1120" yWindow="600" windowWidth="50080" windowHeight="28200" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="81" r:id="rId1"/>
@@ -65,9 +65,6 @@
     <t>numScenarios</t>
   </si>
   <si>
-    <t>Total Cost (4-h System), [$/KWh]</t>
-  </si>
-  <si>
     <t>Low Scenario</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
     <t>E, [€, MWh]</t>
   </si>
   <si>
-    <t>Total Cost (4-h System), [€/KWh]</t>
-  </si>
-  <si>
     <t>Scenario 1</t>
   </si>
   <si>
@@ -129,6 +123,12 @@
   </si>
   <si>
     <t>Scenario 3</t>
+  </si>
+  <si>
+    <t>Total Cost (4-h System), [€/kW]</t>
+  </si>
+  <si>
+    <t>Total Cost (4-h System), [$/kW]</t>
   </si>
 </sst>
 </file>
@@ -484,9 +484,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14E7A88E-2477-46FD-BE5E-2BB647C1CD4A}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -511,19 +511,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7614B8E9-E001-4C19-AEEE-8FBC4B48A529}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" s="4">
         <f>C2</f>
@@ -541,79 +541,79 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24F6E267-467C-483D-8CCD-C38B5B3B7274}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>270.22000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>5.69</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>20.94</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>11.73</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>44.84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7">
         <v>23.09</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>10.95</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9">
         <v>24.38</v>
@@ -628,14 +628,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1BF002-C479-4585-BB53-0E4A987995C6}">
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -731,9 +731,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="3">
         <v>1587.252</v>
@@ -829,9 +829,9 @@
         <v>588.10199999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3">
         <v>1587.252</v>
@@ -927,9 +927,9 @@
         <v>832.64599999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3">
         <v>1587.252</v>
@@ -1033,14 +1033,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A2E7FA-B63A-489C-AACF-5835B538C347}">
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -1136,9 +1136,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="3">
         <f>'Investment Cost NREL, USD'!B2/'Conversion rate'!$B$2</f>
@@ -1265,9 +1265,9 @@
         <v>543.58258619096023</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3">
         <f>'Investment Cost NREL, USD'!B3/'Conversion rate'!$B$2</f>
@@ -1394,9 +1394,9 @@
         <v>769.61456696552352</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3">
         <f>'Investment Cost NREL, USD'!B4/'Conversion rate'!$B$2</f>
@@ -1531,27 +1531,27 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2823AF14-4748-4019-BD7D-F91F970D3C5E}">
   <dimension ref="A1:AJ5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="10.5546875" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="9.5546875" customWidth="1"/>
-    <col min="17" max="17" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="21" width="9.5546875" customWidth="1"/>
-    <col min="22" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="26" width="9.5546875" customWidth="1"/>
-    <col min="27" max="27" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="31" width="9.5546875" customWidth="1"/>
-    <col min="32" max="36" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="10.5" customWidth="1"/>
+    <col min="12" max="12" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="16" width="9.5" customWidth="1"/>
+    <col min="17" max="17" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="21" width="9.5" customWidth="1"/>
+    <col min="22" max="22" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="9.5" customWidth="1"/>
+    <col min="27" max="27" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="28" max="31" width="9.5" customWidth="1"/>
+    <col min="32" max="36" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -1659,9 +1659,9 @@
         <v>2054</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B2" s="2">
         <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)*1000*('Cost breakdown NREL'!$B$9+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
@@ -1800,9 +1800,9 @@
         <v>109550.68631956511</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2">
         <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)*1000*('Cost breakdown NREL'!$B$9+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
@@ -1941,9 +1941,9 @@
         <v>155103.94584823828</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="2">
         <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)*1000*('Cost breakdown NREL'!$B$9+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
@@ -2082,7 +2082,7 @@
         <v>240015.5911859858</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="F5" s="2"/>
@@ -2096,27 +2096,27 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75013386-D65F-4F42-82AA-9369535BE7EB}">
   <dimension ref="A1:AJ4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="10.5546875" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="9.5546875" customWidth="1"/>
-    <col min="17" max="17" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="21" width="9.5546875" customWidth="1"/>
-    <col min="22" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="26" width="9.5546875" customWidth="1"/>
-    <col min="27" max="27" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="31" width="9.5546875" customWidth="1"/>
-    <col min="32" max="36" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="10.5" customWidth="1"/>
+    <col min="12" max="12" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="16" width="9.5" customWidth="1"/>
+    <col min="17" max="17" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="21" width="9.5" customWidth="1"/>
+    <col min="22" max="22" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="9.5" customWidth="1"/>
+    <col min="27" max="27" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="28" max="31" width="9.5" customWidth="1"/>
+    <col min="32" max="36" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1">
         <v>2020</v>
@@ -2224,427 +2224,427 @@
         <v>2054</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2">
+        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
+      </c>
+      <c r="C2" s="2">
+        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
+      </c>
+      <c r="D2" s="2">
+        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>329157.57358866697</v>
+      </c>
+      <c r="E2" s="2">
+        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>236795.84773646726</v>
+      </c>
+      <c r="F2" s="2">
+        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>223504.08114379484</v>
+      </c>
+      <c r="G2" s="2">
+        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>212132.83090957787</v>
+      </c>
+      <c r="H2" s="2">
+        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>203128.6000204107</v>
+      </c>
+      <c r="I2" s="2">
+        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>194124.36913124358</v>
+      </c>
+      <c r="J2" s="2">
+        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>185120.13824207647</v>
+      </c>
+      <c r="K2" s="2">
+        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>176115.53834217665</v>
+      </c>
+      <c r="L2" s="2">
+        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>167114.25953887129</v>
+      </c>
+      <c r="M2" s="2">
+        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>164184.12981568652</v>
+      </c>
+      <c r="N2" s="2">
+        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>161254.00009250178</v>
+      </c>
+      <c r="O2" s="2">
+        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>158321.10278882159</v>
+      </c>
+      <c r="P2" s="2">
+        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>155391.15757100319</v>
+      </c>
+      <c r="Q2" s="2">
+        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>152464.16443904658</v>
+      </c>
+      <c r="R2" s="2">
+        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>149531.08263000002</v>
+      </c>
+      <c r="S2" s="2">
+        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>146601.13741218162</v>
+      </c>
+      <c r="T2" s="2">
+        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>143671.00768899688</v>
+      </c>
+      <c r="U2" s="2">
+        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>140741.06247117848</v>
+      </c>
+      <c r="V2" s="2">
+        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>137807.98066213191</v>
+      </c>
+      <c r="W2" s="2">
+        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>134878.03544431349</v>
+      </c>
+      <c r="X2" s="2">
+        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>131951.04231235688</v>
+      </c>
+      <c r="Y2" s="2">
+        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>129021.09709453849</v>
+      </c>
+      <c r="Z2" s="2">
+        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>126088.01528549194</v>
+      </c>
+      <c r="AA2" s="2">
+        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>123157.88556230719</v>
+      </c>
+      <c r="AB2" s="2">
+        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>120227.9403444888</v>
+      </c>
+      <c r="AC2" s="2">
+        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>117297.810621304</v>
+      </c>
+      <c r="AD2" s="2">
+        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>114364.72881225747</v>
+      </c>
+      <c r="AE2" s="2">
+        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>111434.78359443907</v>
+      </c>
+      <c r="AF2" s="2">
+        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>108507.97496784879</v>
+      </c>
+      <c r="AG2" s="5">
+        <v>108507.97496784879</v>
+      </c>
+      <c r="AH2" s="5">
+        <v>108507.97496784879</v>
+      </c>
+      <c r="AI2" s="5">
+        <v>108507.97496784879</v>
+      </c>
+      <c r="AJ2" s="5">
+        <v>108507.97496784879</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2">
+        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
+      </c>
+      <c r="C3" s="2">
+        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
+      </c>
+      <c r="D3" s="2">
+        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>329157.57358866697</v>
+      </c>
+      <c r="E3" s="2">
+        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>316519.32500364655</v>
+      </c>
+      <c r="F3" s="2">
+        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>302362.78175883851</v>
+      </c>
+      <c r="G3" s="2">
+        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>264982.36354475952</v>
+      </c>
+      <c r="H3" s="2">
+        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>256410.4287289771</v>
+      </c>
+      <c r="I3" s="2">
+        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>247837.9403970956</v>
+      </c>
+      <c r="J3" s="2">
+        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>239264.71404374859</v>
+      </c>
+      <c r="K3" s="2">
+        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>230690.74966893613</v>
+      </c>
+      <c r="L3" s="2">
+        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>222115.86276729195</v>
+      </c>
+      <c r="M3" s="2">
+        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>218690.15163006057</v>
+      </c>
+      <c r="N3" s="2">
+        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>215264.62499819553</v>
+      </c>
+      <c r="O3" s="2">
+        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>211839.09836633052</v>
+      </c>
+      <c r="P3" s="2">
+        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>208413.57173446551</v>
+      </c>
+      <c r="Q3" s="2">
+        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>204988.41411333327</v>
+      </c>
+      <c r="R3" s="2">
+        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>201563.25649220095</v>
+      </c>
+      <c r="S3" s="2">
+        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>198138.09887106865</v>
+      </c>
+      <c r="T3" s="2">
+        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>194713.31026066907</v>
+      </c>
+      <c r="U3" s="2">
+        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>191288.52165026945</v>
+      </c>
+      <c r="V3" s="2">
+        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>187863.91754523627</v>
+      </c>
+      <c r="W3" s="2">
+        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>184439.49794556946</v>
+      </c>
+      <c r="X3" s="2">
+        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>181015.26285126893</v>
+      </c>
+      <c r="Y3" s="2">
+        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>177591.2122623348</v>
+      </c>
+      <c r="Z3" s="2">
+        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>174167.1616734007</v>
+      </c>
+      <c r="AA3" s="2">
+        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>170743.48009519925</v>
+      </c>
+      <c r="AB3" s="2">
+        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>167319.79851699786</v>
+      </c>
+      <c r="AC3" s="2">
+        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>163896.48594952916</v>
+      </c>
+      <c r="AD3" s="2">
+        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>160473.35788742686</v>
+      </c>
+      <c r="AE3" s="2">
+        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>157050.41433069092</v>
+      </c>
+      <c r="AF3" s="2">
+        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>153627.6552793213</v>
+      </c>
+      <c r="AG3" s="5">
+        <v>153627.6552793213</v>
+      </c>
+      <c r="AH3" s="5">
+        <v>153627.6552793213</v>
+      </c>
+      <c r="AI3" s="5">
+        <v>153627.6552793213</v>
+      </c>
+      <c r="AJ3" s="5">
+        <v>153627.6552793213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="2">
-        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
-      </c>
-      <c r="C2" s="2">
-        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
-      </c>
-      <c r="D2" s="2">
-        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>263326.05887093366</v>
-      </c>
-      <c r="E2" s="2">
-        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>189436.67818917381</v>
-      </c>
-      <c r="F2" s="2">
-        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>178803.26491503586</v>
-      </c>
-      <c r="G2" s="2">
-        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>169706.26472766226</v>
-      </c>
-      <c r="H2" s="2">
-        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>162502.88001632856</v>
-      </c>
-      <c r="I2" s="2">
-        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>155299.49530499487</v>
-      </c>
-      <c r="J2" s="2">
-        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>148096.11059366117</v>
-      </c>
-      <c r="K2" s="2">
-        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>140892.43067374133</v>
-      </c>
-      <c r="L2" s="2">
-        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>133691.40763109707</v>
-      </c>
-      <c r="M2" s="2">
-        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>131347.30385254926</v>
-      </c>
-      <c r="N2" s="2">
-        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>129003.20007400145</v>
-      </c>
-      <c r="O2" s="2">
-        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>126656.88223105727</v>
-      </c>
-      <c r="P2" s="2">
-        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>124312.92605680255</v>
-      </c>
-      <c r="Q2" s="2">
-        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>121971.33155123725</v>
-      </c>
-      <c r="R2" s="2">
-        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>119624.86610400002</v>
-      </c>
-      <c r="S2" s="2">
-        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>117280.90992974529</v>
-      </c>
-      <c r="T2" s="2">
-        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>114936.80615119748</v>
-      </c>
-      <c r="U2" s="2">
-        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>112592.84997694279</v>
-      </c>
-      <c r="V2" s="2">
-        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>110246.38452970554</v>
-      </c>
-      <c r="W2" s="2">
-        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>107902.42835545079</v>
-      </c>
-      <c r="X2" s="2">
-        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>105560.8338498855</v>
-      </c>
-      <c r="Y2" s="2">
-        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>103216.87767563078</v>
-      </c>
-      <c r="Z2" s="2">
-        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>100870.41222839357</v>
-      </c>
-      <c r="AA2" s="2">
-        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>98526.308449845747</v>
-      </c>
-      <c r="AB2" s="2">
-        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>96182.352275591023</v>
-      </c>
-      <c r="AC2" s="2">
-        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>93838.248497043183</v>
-      </c>
-      <c r="AD2" s="2">
-        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>91491.783049805977</v>
-      </c>
-      <c r="AE2" s="2">
-        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>89147.826875551254</v>
-      </c>
-      <c r="AF2" s="2">
-        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,2,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>86806.379974279029</v>
-      </c>
-      <c r="AG2" s="5">
-        <v>86806.379974279029</v>
-      </c>
-      <c r="AH2" s="5">
-        <v>86806.379974279029</v>
-      </c>
-      <c r="AI2" s="5">
-        <v>86806.379974279029</v>
-      </c>
-      <c r="AJ2" s="5">
-        <v>86806.379974279029</v>
-      </c>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="2">
-        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
-      </c>
-      <c r="C3" s="2">
-        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
-      </c>
-      <c r="D3" s="2">
-        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>263326.05887093366</v>
-      </c>
-      <c r="E3" s="2">
-        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>253215.46000291719</v>
-      </c>
-      <c r="F3" s="2">
-        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>241890.22540707077</v>
-      </c>
-      <c r="G3" s="2">
-        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>211985.89083580763</v>
-      </c>
-      <c r="H3" s="2">
-        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>205128.34298318165</v>
-      </c>
-      <c r="I3" s="2">
-        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>198270.35231767647</v>
-      </c>
-      <c r="J3" s="2">
-        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>191411.77123499889</v>
-      </c>
-      <c r="K3" s="2">
-        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>184552.59973514895</v>
-      </c>
-      <c r="L3" s="2">
-        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>177692.69021383356</v>
-      </c>
-      <c r="M3" s="2">
-        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>174952.12130404849</v>
-      </c>
-      <c r="N3" s="2">
-        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>172211.69999855643</v>
-      </c>
-      <c r="O3" s="2">
-        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>169471.27869306441</v>
-      </c>
-      <c r="P3" s="2">
-        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>166730.85738757241</v>
-      </c>
-      <c r="Q3" s="2">
-        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>163990.73129066662</v>
-      </c>
-      <c r="R3" s="2">
-        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>161250.60519376074</v>
-      </c>
-      <c r="S3" s="2">
-        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>158510.47909685489</v>
-      </c>
-      <c r="T3" s="2">
-        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>155770.64820853525</v>
-      </c>
-      <c r="U3" s="2">
-        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>153030.81732021557</v>
-      </c>
-      <c r="V3" s="2">
-        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>150291.13403618903</v>
-      </c>
-      <c r="W3" s="2">
-        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>147551.59835645556</v>
-      </c>
-      <c r="X3" s="2">
-        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>144812.21028101514</v>
-      </c>
-      <c r="Y3" s="2">
-        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>142072.96980986785</v>
-      </c>
-      <c r="Z3" s="2">
-        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>139333.72933872056</v>
-      </c>
-      <c r="AA3" s="2">
-        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>136594.78407615941</v>
-      </c>
-      <c r="AB3" s="2">
-        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>133855.8388135983</v>
-      </c>
-      <c r="AC3" s="2">
-        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>131117.18875962336</v>
-      </c>
-      <c r="AD3" s="2">
-        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>128378.68630994151</v>
-      </c>
-      <c r="AE3" s="2">
-        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>125640.33146455274</v>
-      </c>
-      <c r="AF3" s="2">
-        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,3,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>122902.12422345704</v>
-      </c>
-      <c r="AG3" s="5">
-        <v>122902.12422345704</v>
-      </c>
-      <c r="AH3" s="5">
-        <v>122902.12422345704</v>
-      </c>
-      <c r="AI3" s="5">
-        <v>122902.12422345704</v>
-      </c>
-      <c r="AJ3" s="5">
-        <v>122902.12422345704</v>
-      </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
       <c r="B4" s="2">
-        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
+        <f>HLOOKUP(B$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
       </c>
       <c r="C4" s="2">
-        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>234285.20941424163</v>
+        <f>HLOOKUP(C$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>292856.51176780206</v>
       </c>
       <c r="D4" s="2">
-        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>263326.05887093366</v>
+        <f>HLOOKUP(D$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>329157.57358866697</v>
       </c>
       <c r="E4" s="2">
-        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>273079.75055826054</v>
+        <f>HLOOKUP(E$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>341349.68819782574</v>
       </c>
       <c r="F4" s="2">
-        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>275029.30806138122</v>
+        <f>HLOOKUP(F$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>343786.63507672655</v>
       </c>
       <c r="G4" s="2">
-        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>271127.09336498502</v>
+        <f>HLOOKUP(G$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>338908.86670623126</v>
       </c>
       <c r="H4" s="2">
-        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>260973.39404338662</v>
+        <f>HLOOKUP(H$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>326216.74255423329</v>
       </c>
       <c r="I4" s="2">
-        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>250819.8423260813</v>
+        <f>HLOOKUP(I$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>313524.80290760164</v>
       </c>
       <c r="J4" s="2">
-        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>240666.43821306911</v>
+        <f>HLOOKUP(J$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>300833.04776633636</v>
       </c>
       <c r="K4" s="2">
-        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>230513.18170434996</v>
+        <f>HLOOKUP(K$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>288141.4771304375</v>
       </c>
       <c r="L4" s="2">
-        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>220360.07279992398</v>
+        <f>HLOOKUP(L$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>275450.09099990502</v>
       </c>
       <c r="M4" s="2">
-        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>218851.4093202604</v>
+        <f>HLOOKUP(M$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>273564.2616503255</v>
       </c>
       <c r="N4" s="2">
-        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>217342.59823630378</v>
+        <f>HLOOKUP(N$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>271678.24779537966</v>
       </c>
       <c r="O4" s="2">
-        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>215833.7871523471</v>
+        <f>HLOOKUP(O$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>269792.23394043389</v>
       </c>
       <c r="P4" s="2">
-        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>214325.12367268346</v>
+        <f>HLOOKUP(P$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>267906.40459085436</v>
       </c>
       <c r="Q4" s="2">
-        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>212816.31258872684</v>
+        <f>HLOOKUP(Q$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>266020.39073590853</v>
       </c>
       <c r="R4" s="2">
-        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>211307.50150477022</v>
+        <f>HLOOKUP(R$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>264134.37688096275</v>
       </c>
       <c r="S4" s="2">
-        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>209798.83802510661</v>
+        <f>HLOOKUP(S$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>262248.54753138323</v>
       </c>
       <c r="T4" s="2">
-        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>208290.02694114993</v>
+        <f>HLOOKUP(T$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>260362.53367643742</v>
       </c>
       <c r="U4" s="2">
-        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>206781.36346148638</v>
+        <f>HLOOKUP(U$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>258476.70432685793</v>
       </c>
       <c r="V4" s="2">
-        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>205272.5523775297</v>
+        <f>HLOOKUP(V$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>256590.69047191215</v>
       </c>
       <c r="W4" s="2">
-        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>203763.74129357305</v>
+        <f>HLOOKUP(W$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>254704.67661696632</v>
       </c>
       <c r="X4" s="2">
-        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>202255.07781390948</v>
+        <f>HLOOKUP(X$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>252818.84726738679</v>
       </c>
       <c r="Y4" s="2">
-        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>200746.26672995285</v>
+        <f>HLOOKUP(Y$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>250932.83341244105</v>
       </c>
       <c r="Z4" s="2">
-        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>199237.45564599618</v>
+        <f>HLOOKUP(Z$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>249046.81955749524</v>
       </c>
       <c r="AA4" s="2">
-        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>197728.79216633263</v>
+        <f>HLOOKUP(AA$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>247160.99020791572</v>
       </c>
       <c r="AB4" s="2">
-        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>196219.98108237592</v>
+        <f>HLOOKUP(AB$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>245274.97635296991</v>
       </c>
       <c r="AC4" s="2">
-        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>194711.16999841927</v>
+        <f>HLOOKUP(AC$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>243388.96249802408</v>
       </c>
       <c r="AD4" s="2">
-        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>193202.50651875572</v>
+        <f>HLOOKUP(AD$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>241503.13314844461</v>
       </c>
       <c r="AE4" s="2">
-        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>191693.69543479901</v>
+        <f>HLOOKUP(AE$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>239617.11929349878</v>
       </c>
       <c r="AF4" s="2">
-        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/5*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
-        <v>190184.88435084239</v>
+        <f>HLOOKUP(AF$1,'Investment Cost NREL, EUR'!$B$1:$AF$4,4,FALSE)/4*1000*('Cost breakdown NREL'!$B$2+SUM('Cost breakdown NREL'!$B$3:$B$8)/2)/SUM('Cost breakdown NREL'!$B$2:$B$9)</f>
+        <v>237731.10543855297</v>
       </c>
       <c r="AG4" s="5">
-        <v>190184.88435084239</v>
+        <v>237731.10543855297</v>
       </c>
       <c r="AH4" s="5">
-        <v>190184.88435084239</v>
+        <v>237731.10543855297</v>
       </c>
       <c r="AI4" s="5">
-        <v>190184.88435084239</v>
+        <v>237731.10543855297</v>
       </c>
       <c r="AJ4" s="5">
-        <v>190184.88435084239</v>
+        <v>237731.10543855297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>